<commit_message>
[update] => summary format number and create popup success message for insert success
</commit_message>
<xml_diff>
--- a/public/excel/2025-3-PurchaseList.xlsx
+++ b/public/excel/2025-3-PurchaseList.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,7 +416,7 @@
         <v>price</v>
       </c>
       <c r="F1" t="str">
-        <v>materialPrice</v>
+        <v>costPrice</v>
       </c>
       <c r="G1" t="str">
         <v>gpPrice</v>
@@ -433,25 +433,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>A02</v>
+        <v>A01</v>
       </c>
       <c r="C2" t="str">
-        <v>ยำทะเล</v>
+        <v>ยำวุ้นเส้น</v>
       </c>
       <c r="D2" t="str">
-        <v xml:space="preserve">            </v>
+        <v>หมูสับ (100กรัม)</v>
       </c>
       <c r="E2">
-        <v>100</v>
-      </c>
-      <c r="F2">
-        <v>45</v>
-      </c>
-      <c r="G2">
-        <v>30</v>
-      </c>
-      <c r="H2">
-        <v>18</v>
+        <v>110</v>
+      </c>
+      <c r="F2" t="str">
+        <v>44.00</v>
+      </c>
+      <c r="G2" t="str">
+        <v>35.31</v>
+      </c>
+      <c r="H2" t="str">
+        <v>30.69</v>
       </c>
       <c r="I2" t="str">
         <v>GrabFood</v>
@@ -462,28 +462,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>A02</v>
+        <v>A01</v>
       </c>
       <c r="C3" t="str">
-        <v>ยำทะเล</v>
+        <v>ยำวุ้นเส้น</v>
       </c>
       <c r="D3" t="str">
-        <v xml:space="preserve">            </v>
+        <v>ข้าวสวย</v>
       </c>
       <c r="E3">
-        <v>100</v>
-      </c>
-      <c r="F3">
-        <v>45</v>
-      </c>
-      <c r="G3">
-        <v>30</v>
-      </c>
-      <c r="H3">
-        <v>18</v>
+        <v>105</v>
+      </c>
+      <c r="F3" t="str">
+        <v>42.00</v>
+      </c>
+      <c r="G3" t="str">
+        <v>33.70</v>
+      </c>
+      <c r="H3" t="str">
+        <v>29.30</v>
       </c>
       <c r="I3" t="str">
-        <v>GrabFood</v>
+        <v>LineManFood</v>
       </c>
     </row>
     <row r="4">
@@ -491,28 +491,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>A02</v>
+        <v>A05</v>
       </c>
       <c r="C4" t="str">
         <v>ยำทะเล</v>
       </c>
       <c r="D4" t="str">
-        <v xml:space="preserve">            </v>
+        <v>ปลาหมึก (100กรัม)</v>
       </c>
       <c r="E4">
-        <v>100</v>
-      </c>
-      <c r="F4">
-        <v>45</v>
-      </c>
-      <c r="G4">
-        <v>30</v>
-      </c>
-      <c r="H4">
-        <v>18</v>
+        <v>150</v>
+      </c>
+      <c r="F4" t="str">
+        <v>60.00</v>
+      </c>
+      <c r="G4" t="str">
+        <v>48.15</v>
+      </c>
+      <c r="H4" t="str">
+        <v>41.85</v>
       </c>
       <c r="I4" t="str">
-        <v>GrabFood</v>
+        <v>LineManFood</v>
       </c>
     </row>
     <row r="5">
@@ -520,25 +520,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>A02</v>
+        <v>A01</v>
       </c>
       <c r="C5" t="str">
-        <v>ยำทะเล</v>
+        <v>ยำวุ้นเส้น</v>
       </c>
       <c r="D5" t="str">
-        <v xml:space="preserve">            </v>
+        <v>หมูสับ (100กรัม),หมูยอ (100กรัม)</v>
       </c>
       <c r="E5">
-        <v>100</v>
-      </c>
-      <c r="F5">
-        <v>45</v>
-      </c>
-      <c r="G5">
-        <v>30</v>
-      </c>
-      <c r="H5">
-        <v>18</v>
+        <v>130</v>
+      </c>
+      <c r="F5" t="str">
+        <v>52.00</v>
+      </c>
+      <c r="G5" t="str">
+        <v>41.73</v>
+      </c>
+      <c r="H5" t="str">
+        <v>36.27</v>
       </c>
       <c r="I5" t="str">
         <v>GrabFood</v>
@@ -549,25 +549,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>A02</v>
+        <v>A07</v>
       </c>
       <c r="C6" t="str">
-        <v>ยำทะเล</v>
+        <v>ข้าวคลุกกะเพราหมูสับ</v>
       </c>
       <c r="D6" t="str">
-        <v xml:space="preserve">            </v>
+        <v>ข้าวสวย</v>
       </c>
       <c r="E6">
-        <v>100</v>
-      </c>
-      <c r="F6">
-        <v>45</v>
-      </c>
-      <c r="G6">
-        <v>30</v>
-      </c>
-      <c r="H6">
-        <v>18</v>
+        <v>95</v>
+      </c>
+      <c r="F6" t="str">
+        <v>38.00</v>
+      </c>
+      <c r="G6" t="str">
+        <v>30.50</v>
+      </c>
+      <c r="H6" t="str">
+        <v>26.50</v>
       </c>
       <c r="I6" t="str">
         <v>GrabFood</v>
@@ -578,28 +578,28 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>A01</v>
+        <v>A10</v>
       </c>
       <c r="C7" t="str">
-        <v>ยำหมูสับ</v>
+        <v>ข้าวไข่เจียวแหนม (ไข่ 2 ฟอง)</v>
       </c>
       <c r="D7" t="str">
-        <v xml:space="preserve">            </v>
+        <v>หมูสับ (100กรัม),กุ้ง (3ตัว)</v>
       </c>
       <c r="E7">
-        <v>80</v>
-      </c>
-      <c r="F7">
-        <v>35</v>
-      </c>
-      <c r="G7">
-        <v>24</v>
-      </c>
-      <c r="H7">
-        <v>15.4</v>
+        <v>105</v>
+      </c>
+      <c r="F7" t="str">
+        <v>42.00</v>
+      </c>
+      <c r="G7" t="str">
+        <v>33.70</v>
+      </c>
+      <c r="H7" t="str">
+        <v>29.30</v>
       </c>
       <c r="I7" t="str">
-        <v>GrabFood</v>
+        <v>LineManFood</v>
       </c>
     </row>
     <row r="8">
@@ -607,25 +607,25 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>A01</v>
+        <v>A03</v>
       </c>
       <c r="C8" t="str">
-        <v>ยำหมูสับ</v>
+        <v>ยำมาม่า</v>
       </c>
       <c r="D8" t="str">
-        <v xml:space="preserve">            </v>
+        <v>หมูสับ (100กรัม),หมูยอ (100กรัม),หมูสับ (100กรัม)</v>
       </c>
       <c r="E8">
-        <v>80</v>
-      </c>
-      <c r="F8">
-        <v>35</v>
-      </c>
-      <c r="G8">
-        <v>24</v>
-      </c>
-      <c r="H8">
-        <v>15.4</v>
+        <v>150</v>
+      </c>
+      <c r="F8" t="str">
+        <v>60.00</v>
+      </c>
+      <c r="G8" t="str">
+        <v>48.15</v>
+      </c>
+      <c r="H8" t="str">
+        <v>41.85</v>
       </c>
       <c r="I8" t="str">
         <v>GrabFood</v>
@@ -636,28 +636,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>A01</v>
+        <v>A05</v>
       </c>
       <c r="C9" t="str">
-        <v>ยำหมูสับ</v>
+        <v>ยำทะเล</v>
       </c>
       <c r="D9" t="str">
-        <v xml:space="preserve">            </v>
+        <v>ไข่ดาว</v>
       </c>
       <c r="E9">
-        <v>80</v>
-      </c>
-      <c r="F9">
-        <v>35</v>
-      </c>
-      <c r="G9">
-        <v>24</v>
-      </c>
-      <c r="H9">
-        <v>15.4</v>
+        <v>145</v>
+      </c>
+      <c r="F9" t="str">
+        <v>58.00</v>
+      </c>
+      <c r="G9" t="str">
+        <v>46.55</v>
+      </c>
+      <c r="H9" t="str">
+        <v>40.45</v>
       </c>
       <c r="I9" t="str">
-        <v>GrabFood</v>
+        <v>LineManFood</v>
       </c>
     </row>
     <row r="10">
@@ -665,28 +665,28 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>A01</v>
+        <v>A02</v>
       </c>
       <c r="C10" t="str">
         <v>ยำหมูสับ</v>
       </c>
       <c r="D10" t="str">
-        <v xml:space="preserve">            </v>
+        <v>หมูยอ (100กรัม)</v>
       </c>
       <c r="E10">
-        <v>80</v>
-      </c>
-      <c r="F10">
-        <v>35</v>
-      </c>
-      <c r="G10">
-        <v>24</v>
-      </c>
-      <c r="H10">
-        <v>15.4</v>
+        <v>120</v>
+      </c>
+      <c r="F10" t="str">
+        <v>48.00</v>
+      </c>
+      <c r="G10" t="str">
+        <v>38.52</v>
+      </c>
+      <c r="H10" t="str">
+        <v>33.48</v>
       </c>
       <c r="I10" t="str">
-        <v>GrabFood</v>
+        <v>LineManFood</v>
       </c>
     </row>
     <row r="11">
@@ -694,28 +694,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>A03</v>
+        <v>A11</v>
       </c>
       <c r="C11" t="str">
-        <v>ยำมาม่า</v>
+        <v>ข้าวหน้าไข่กะทะ (ไข่ 2 ฟอง)</v>
       </c>
       <c r="D11" t="str">
-        <v>ไข่เจียว,ไข่ดาว,กุ้ง (3ตัว),ปลาหมึก (100กรัม),หมูยอ (100กรัม)</v>
+        <v>กุ้ง (3ตัว)</v>
       </c>
       <c r="E11">
-        <v>180</v>
-      </c>
-      <c r="F11">
-        <v>72</v>
-      </c>
-      <c r="G11">
-        <v>57.78</v>
-      </c>
-      <c r="H11">
-        <v>50.22</v>
+        <v>85</v>
+      </c>
+      <c r="F11" t="str">
+        <v>34.00</v>
+      </c>
+      <c r="G11" t="str">
+        <v>27.29</v>
+      </c>
+      <c r="H11" t="str">
+        <v>23.71</v>
       </c>
       <c r="I11" t="str">
-        <v>LineManFood</v>
+        <v>GrabFood</v>
       </c>
     </row>
     <row r="12">
@@ -723,25 +723,25 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>A05</v>
+        <v>A02</v>
       </c>
       <c r="C12" t="str">
-        <v>ยำทะเล</v>
+        <v>ยำหมูสับ</v>
       </c>
       <c r="D12" t="str">
-        <v>หมูยอ (100กรัม),ข้าวสวย,ปลาหมึก (100กรัม),กุ้ง (3ตัว)</v>
+        <v>หมูสับ (100กรัม)</v>
       </c>
       <c r="E12">
-        <v>205</v>
-      </c>
-      <c r="F12">
-        <v>82</v>
-      </c>
-      <c r="G12">
-        <v>65.805</v>
-      </c>
-      <c r="H12">
-        <v>57.19499999999999</v>
+        <v>120</v>
+      </c>
+      <c r="F12" t="str">
+        <v>48.00</v>
+      </c>
+      <c r="G12" t="str">
+        <v>38.52</v>
+      </c>
+      <c r="H12" t="str">
+        <v>33.48</v>
       </c>
       <c r="I12" t="str">
         <v>GrabFood</v>
@@ -752,33 +752,149 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>A08</v>
+        <v>A01</v>
       </c>
       <c r="C13" t="str">
-        <v>ข้าวไข่เจียว (ไข่ 2 ฟอง)</v>
+        <v>ยำวุ้นเส้น</v>
       </c>
       <c r="D13" t="str">
-        <v>หมูยอ (100กรัม),ข้าวสวย,ปลาหมึก (100กรัม),กุ้ง (3ตัว)</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="E13">
-        <v>150</v>
-      </c>
-      <c r="F13">
-        <v>60</v>
-      </c>
-      <c r="G13">
-        <v>48.15</v>
-      </c>
-      <c r="H13">
-        <v>41.85</v>
+        <v>90</v>
+      </c>
+      <c r="F13" t="str">
+        <v>36.00</v>
+      </c>
+      <c r="G13" t="str">
+        <v>28.89</v>
+      </c>
+      <c r="H13" t="str">
+        <v>25.11</v>
       </c>
       <c r="I13" t="str">
         <v>GrabFood</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>A01</v>
+      </c>
+      <c r="C14" t="str">
+        <v>ยำวุ้นเส้น</v>
+      </c>
+      <c r="D14" t="str">
+        <v>หมูสับ (100กรัม)</v>
+      </c>
+      <c r="E14">
+        <v>110</v>
+      </c>
+      <c r="F14" t="str">
+        <v>44.00</v>
+      </c>
+      <c r="G14" t="str">
+        <v>35.31</v>
+      </c>
+      <c r="H14" t="str">
+        <v>30.69</v>
+      </c>
+      <c r="I14" t="str">
+        <v>LineManFood</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>A02</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ยำหมูสับ</v>
+      </c>
+      <c r="D15" t="str">
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="E15">
+        <v>100</v>
+      </c>
+      <c r="F15" t="str">
+        <v>40.00</v>
+      </c>
+      <c r="G15" t="str">
+        <v>32.10</v>
+      </c>
+      <c r="H15" t="str">
+        <v>27.90</v>
+      </c>
+      <c r="I15" t="str">
+        <v>GrabFood</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>A04</v>
+      </c>
+      <c r="C16" t="str">
+        <v>ยำหมููยอ</v>
+      </c>
+      <c r="D16" t="str">
+        <v>ปลาหมึก (100กรัม)</v>
+      </c>
+      <c r="E16">
+        <v>130</v>
+      </c>
+      <c r="F16" t="str">
+        <v>52.00</v>
+      </c>
+      <c r="G16" t="str">
+        <v>41.73</v>
+      </c>
+      <c r="H16" t="str">
+        <v>36.27</v>
+      </c>
+      <c r="I16" t="str">
+        <v>GrabFood</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>A04</v>
+      </c>
+      <c r="C17" t="str">
+        <v>ยำหมููยอ</v>
+      </c>
+      <c r="D17" t="str">
+        <v>หมูยอ (100กรัม)</v>
+      </c>
+      <c r="E17">
+        <v>110</v>
+      </c>
+      <c r="F17" t="str">
+        <v>44.00</v>
+      </c>
+      <c r="G17" t="str">
+        <v>35.31</v>
+      </c>
+      <c r="H17" t="str">
+        <v>30.69</v>
+      </c>
+      <c r="I17" t="str">
+        <v>GrabFood</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>